<commit_message>
kccn-sct-vn v1.17.0: KCN Phu Xuan + Phu Xuan 1 duoc phe duyet Dieu chinh cuc bo QHPK (QD 129 + 130/QD-BQL ngay 06/8/2026, Truong ban Vuong Trinh Quoc ky; XLNT chung 45.000 m3/ngd tai Phu Xuan; nha may nuoc 70.000 m3/ngd tai Phu Xuan 1; 01 TBA 110kV dung chung) - luu van ban goc + cap nhat ref 26 + 03 file ky 07/8
</commit_message>
<xml_diff>
--- a/kccn-sct-vn/skills/kccn-sct-vn/vi-du-thuc-te/2026.08.07. Theo dõi tiến độ CCN, KCN và nhiệm vụ triển khai ngay (bản in A4 ngang).xlsx
+++ b/kccn-sct-vn/skills/kccn-sct-vn/vi-du-thuc-te/2026.08.07. Theo dõi tiến độ CCN, KCN và nhiệm vụ triển khai ngay (bản in A4 ngang).xlsx
@@ -957,7 +957,7 @@
     <row r="65">
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>- Đôn đốc kết quả thẩm định điều chỉnh cục bộ Quy hoạch phân khu Khu công nghiệp Phú Xuân, Phú Xuân 1 (Sở đã tham gia ý kiến tại 4553/SCT-CN ngày 29/7/2026) và phương án cấp điện hai khu (4607/SCT-NL ngày 31/7/2026); đôn đốc thủ tục sau chấp thuận chủ trương đầu tư của 05 khu công nghiệp mới (Bản Qua, Phú Xuân, Phú Xuân 1, Võ Lao, Cam Đường).</t>
+          <t>- Khu công nghiệp Phú Xuân, Phú Xuân 1: Ban Quản lý Khu kinh tế tỉnh đã phê duyệt Điều chỉnh cục bộ Quy hoạch phân khu tại Quyết định 129/QĐ-BQL và 130/QĐ-BQL cùng ngày 06/8/2026 (Trưởng ban Vương Trinh Quốc ký). Nội dung đáng chú ý: nhà máy xử lý nước thải tập trung chung 02 khu công suất 45.000 m3/ngđ đặt tại KCN Phú Xuân; nhà máy nước 70.000 m3/ngđ đặt tại KCN Phú Xuân 1; gộp còn 01 trạm biến áp 110kV (2x63MVA) dùng chung - phù hợp phương án cấp điện Sở đã báo cáo (4607/SCT-NL ngày 31/7/2026). Nhiệm vụ: theo dõi công bố quy hoạch, cắm mốc giới; đôn đốc thủ tục tái định cư, giải phóng mặt bằng, đất đai, môi trường sau điều chỉnh; đôn đốc thủ tục sau chấp thuận chủ trương đầu tư của 05 khu công nghiệp mới (Bản Qua, Phú Xuân, Phú Xuân 1, Võ Lao, Cam Đường).</t>
         </is>
       </c>
     </row>
@@ -2244,18 +2244,21 @@
 - BQL KKT lấy ý kiến điều chỉnh cục bộ QHPK KCN Phú Xuân và Phú Xuân 1: 1125/BQL-QHXD ngày 28/7/2026; Sở đã tham gia ý kiến: 4553/SCT-CN ngày 29/7/2026.
 - NĐT phúc đáp, phối hợp triển khai dự án: 25.7/CV-CNLL ngày 25/7/2026.
 - Sở báo cáo, đề xuất phương án cấp điện KCN Phú Xuân và Phú Xuân 1: 4607/SCT-NL ngày 31/7/2026.
-- Đến 07/8/2026 chưa có kết quả thẩm định hồ sơ điều chỉnh cục bộ QHPK.</t>
+- Quyết định 129/QĐ-BQL ngày 06/8/2026 của Ban Quản lý Khu kinh tế tỉnh (Trưởng ban Vương Trinh Quốc ký) - phê duyệt Điều chỉnh cục bộ Quy hoạch phân khu KCN Phú Xuân (trên cơ sở Tờ trình 32.7/TTr-CNLL ngày 31/7/2026 của nhà đầu tư và Báo cáo thẩm định 39/BC-QHXD ngày 06/8/2026): đất SXCN 183,21 ha còn 175,48 ha (-7,73 ha); Khu XLNT tập trung K2-HTKT1 tăng lên 9,64 ha, quy hoạch nhà máy XLNT chung 02 KCN tổng công suất 45.000 m3/ngđ đặt tại KCN Phú Xuân, đạt cột A QCVN 40:2025/BTNMT; gộp còn 01 TBA 110kV (2x63MVA) tại Phú Xuân cấp điện cho cả 02 KCN.</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>- Theo dõi hồ sơ điều chỉnh cục bộ QHPK.
-- Đôn đốc thủ tục tái định cư, GPMB.</t>
+          <t>- Theo dõi nhà đầu tư công bố quy hoạch, cắm mốc giới sau QĐ 129/QĐ-BQL.
+- Đôn đốc thủ tục tái định cư, GPMB, đất đai, môi trường.
+- Theo dõi triển khai nhà máy XLNT tập trung 45.000 m3/ngđ và TBA 110kV dùng chung 02 KCN.</t>
         </is>
       </c>
       <c r="F12" s="11" t="inlineStr">
         <is>
-          <t>► Đã tham gia ý kiến điều chỉnh cục bộ QHPK (4553/SCT-CN ngày 29/7/2026) – theo dõi kết quả thẩm định; đôn đốc thủ tục tái định cư, GPMB, đất đai, môi trường; theo dõi phương án cấp điện (4607/SCT-NL ngày 31/7/2026).</t>
+          <t>ĐÃ CÓ KẾT QUẢ: BQL Khu kinh tế phê duyệt Điều chỉnh cục bộ QHPK tại QĐ 129/QĐ-BQL ngày 06/8/2026 (Sở đã tham gia ý kiến tại 4553/SCT-CN ngày 29/7/2026; phương án cấp điện tại 4607/SCT-NL ngày 31/7/2026 phù hợp phương án 01 TBA 110kV dùng chung).
+► Theo dõi công bố quy hoạch, cắm mốc giới; đôn đốc thủ tục tái định cư, GPMB sau điều chỉnh.
+► Theo dõi triển khai hạ tầng dùng chung 02 KCN: nhà máy XLNT 45.000 m3/ngđ (đặt tại Phú Xuân), nhà máy nước 70.000 m3/ngđ (đặt tại Phú Xuân 1), TBA 110kV 2x63MVA.</t>
         </is>
       </c>
     </row>
@@ -2284,18 +2287,21 @@
 - Đề nghị điều chỉnh cục bộ QHPK (chung hồ sơ với KCN Phú Xuân): 23.7/2026/CV-LL ngày 23/7/2026.
 - BQL KKT lấy ý kiến điều chỉnh cục bộ QHPK (chung hồ sơ với KCN Phú Xuân): 1125/BQL-QHXD ngày 28/7/2026; Sở đã tham gia ý kiến: 4553/SCT-CN ngày 29/7/2026.
 - Sở báo cáo, đề xuất phương án cấp điện: 4607/SCT-NL ngày 31/7/2026.
-- Đến 07/8/2026 chưa có kết quả thẩm định hồ sơ điều chỉnh cục bộ QHPK.</t>
+- Quyết định 130/QĐ-BQL ngày 06/8/2026 của Ban Quản lý Khu kinh tế tỉnh (Trưởng ban Vương Trinh Quốc ký) - phê duyệt Điều chỉnh cục bộ Quy hoạch phân khu KCN Phú Xuân 1 (Tờ trình 31.7/TTr-CNLL ngày 31/7/2026; Báo cáo thẩm định 40/BC-QHXD ngày 06/8/2026): đất SXCN 118,76 ha tăng lên 126,98 ha (+8,22 ha); bỏ Khu XLNT tại Phú Xuân 1 (xử lý chung tại KCN Phú Xuân), bố trí Trạm cấp nước sạch K1-HTKT1 (5,53 ha) - nhà máy nước công suất 70.000 m3/ngđ cấp cho cả 02 KCN và dân cư lân cận; bổ sung dải cây xanh dọc tuyến kết nối IC17 - ĐT.152.</t>
         </is>
       </c>
       <c r="E13" s="11" t="inlineStr">
         <is>
-          <t>- Theo dõi hồ sơ điều chỉnh cục bộ QHPK.
-- Đôn đốc thủ tục sau CTĐT.</t>
+          <t>- Theo dõi nhà đầu tư công bố quy hoạch, cắm mốc giới sau QĐ 130/QĐ-BQL.
+- Đôn đốc thủ tục sau chấp thuận chủ trương đầu tư.
+- Theo dõi triển khai nhà máy nước 70.000 m3/ngđ cấp cho 02 KCN.</t>
         </is>
       </c>
       <c r="F13" s="11" t="inlineStr">
         <is>
-          <t>► Đã tham gia ý kiến điều chỉnh cục bộ QHPK (4553/SCT-CN ngày 29/7/2026) – theo dõi kết quả thẩm định; đôn đốc thủ tục sau chấp thuận CTĐT.</t>
+          <t>ĐÃ CÓ KẾT QUẢ: BQL Khu kinh tế phê duyệt Điều chỉnh cục bộ QHPK tại QĐ 130/QĐ-BQL ngày 06/8/2026; đất SXCN tăng lên 126,98 ha (63,49%).
+► Theo dõi công bố quy hoạch, cắm mốc giới; đôn đốc thủ tục sau chấp thuận CTĐT.
+► Theo dõi triển khai Trạm cấp nước sạch và nhà máy nước 70.000 m3/ngđ tại Phú Xuân 1 (cấp cho cả 02 KCN và dân cư lân cận).</t>
         </is>
       </c>
     </row>
@@ -3197,7 +3203,8 @@
         <is>
           <t>- Ban Quản lý Khu kinh tế đã hướng dẫn thủ tục sau chấp thuận CTĐT (964/BQL-QHXD ngày 03/7/2026).
 - Khu tái định cư Phú Xuân: UBND tỉnh cho phép lập Báo cáo đề xuất chủ trương đầu tư (7077/UBND-TH ngày 10/7/2026).
-- GPMB: chưa triển khai.</t>
+- GPMB: chưa triển khai.
+- BQL Khu kinh tế đã phê duyệt Điều chỉnh cục bộ QHPK tại QĐ 129/QĐ-BQL ngày 06/8/2026 (XLNT tập trung 45.000 m3/ngđ chung 02 KCN đặt tại Phú Xuân; 01 TBA 110kV 2x63MVA dùng chung).</t>
         </is>
       </c>
       <c r="E12" s="15" t="inlineStr">
@@ -3208,9 +3215,9 @@
       </c>
       <c r="F12" s="15" t="inlineStr">
         <is>
-          <t>Nhà đầu tư đề nghị điều chỉnh cục bộ Quy hoạch phân khu KCN Phú Xuân và Phú Xuân 1 (23.7/2026/CV-LL ngày 23/7/2026); thủ tục tái định cư, GPMB mới ở bước đầu.
-► Theo dõi hồ sơ điều chỉnh cục bộ QHPK; đôn đốc thủ tục tái định cư, GPMB, đất đai, môi trường sau CTĐT.
-► Sở đã tham gia ý kiến điều chỉnh cục bộ QHPK (4553/SCT-CN ngày 29/7/2026) và báo cáo phương án cấp điện (4607/SCT-NL ngày 31/7/2026); NĐT phúc đáp phối hợp triển khai (25.7/CV-CNLL ngày 25/7/2026).</t>
+          <t>ĐÃ phê duyệt Điều chỉnh cục bộ QHPK (QĐ 129/QĐ-BQL ngày 06/8/2026); thủ tục tái định cư, GPMB mới ở bước đầu.
+► Theo dõi công bố quy hoạch, cắm mốc giới; đôn đốc thủ tục tái định cư, GPMB, đất đai, môi trường sau điều chỉnh.
+► Sở đã tham gia ý kiến điều chỉnh (4553/SCT-CN ngày 29/7/2026) và báo cáo phương án cấp điện (4607/SCT-NL ngày 31/7/2026) - phù hợp phương án 01 TBA 110kV dùng chung tại QĐ 129/QĐ-BQL.</t>
         </is>
       </c>
     </row>
@@ -3235,7 +3242,8 @@
       <c r="D13" s="15" t="inlineStr">
         <is>
           <t>- Ban Quản lý Khu kinh tế đã hướng dẫn thủ tục sau chấp thuận CTĐT (965/BQL-QHXD ngày 03/7/2026).
-- GPMB: chưa triển khai.</t>
+- GPMB: chưa triển khai.
+- BQL Khu kinh tế đã phê duyệt Điều chỉnh cục bộ QHPK tại QĐ 130/QĐ-BQL ngày 06/8/2026 (đất SXCN tăng lên 126,98 ha; Trạm cấp nước sạch + nhà máy nước 70.000 m3/ngđ tại Phú Xuân 1 cấp cho 02 KCN).</t>
         </is>
       </c>
       <c r="E13" s="15" t="inlineStr">
@@ -3246,9 +3254,9 @@
       </c>
       <c r="F13" s="15" t="inlineStr">
         <is>
-          <t>Hồ sơ điều chỉnh cục bộ Quy hoạch phân khu chung với KCN Phú Xuân (23.7/2026/CV-LL ngày 23/7/2026).
-► Theo dõi hồ sơ điều chỉnh cục bộ QHPK; đôn đốc thủ tục sau chấp thuận CTĐT.
-► Sở đã tham gia ý kiến điều chỉnh cục bộ QHPK (4553/SCT-CN ngày 29/7/2026) và báo cáo phương án cấp điện (4607/SCT-NL ngày 31/7/2026).</t>
+          <t>ĐÃ phê duyệt Điều chỉnh cục bộ QHPK (QĐ 130/QĐ-BQL ngày 06/8/2026).
+► Theo dõi công bố quy hoạch, cắm mốc giới; đôn đốc thủ tục sau chấp thuận CTĐT.
+► Theo dõi triển khai nhà máy nước 70.000 m3/ngđ và hạ tầng dùng chung 02 KCN.</t>
         </is>
       </c>
     </row>

</xml_diff>